<commit_message>
Feat: Complete TOP 10 promising countries (1 to 10) in Markdown, Word, PPT, Excel and HTML Dashboard
</commit_message>
<xml_diff>
--- a/BIZ-Jeonbok/data/BIZ_Jeonbok_Integrated_Data.xlsx
+++ b/BIZ-Jeonbok/data/BIZ_Jeonbok_Integrated_Data.xlsx
@@ -9,6 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard_Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Size_Pricing_Structure" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top10_Fresh_Abalone" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top10_Frozen_Abalone" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top10_Canned_Abalone" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -30,17 +33,17 @@
       <name val="맑은 고딕"/>
       <b val="1"/>
       <color rgb="001F497D"/>
-      <sz val="16"/>
-    </font>
-    <font>
-      <name val="맑은 고딕"/>
-      <sz val="10"/>
+      <sz val="15"/>
     </font>
     <font>
       <name val="맑은 고딕"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="4">
@@ -89,17 +92,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -467,12 +469,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="87" customWidth="1" min="1" max="1"/>
-    <col width="16.5" customWidth="1" min="2" max="2"/>
-    <col width="40.5" customWidth="1" min="3" max="3"/>
+    <col width="50.4" customWidth="1" min="1" max="1"/>
+    <col width="15.4" customWidth="1" min="2" max="2"/>
+    <col width="37.8" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -482,128 +484,121 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>UN Comtrade 무역 분석 데이터, 미수(Size) 가격 구조 및 로컬 디스트리뷰터 DB 통합 요약</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>핵심 성과 지표 (KPI)</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>측정 수치</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>비고 / 1인 상사 소싱 포인트</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>핵심 성과 지표 (KPI)</t>
+          <t>분석 대상 무역 레코드 수</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>측정 수치</t>
+          <t>500건</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>비고 / 1인 상사 소싱 포인트</t>
+          <t>전 세계 전복 수출입 거래 데이터 정규화</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>분석 대상 무역 레코드 수</t>
+          <t>누적 총 무역액</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>500건</t>
+          <t>$148.50M</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>전 세계 전복 수출입 거래 데이터 정규화</t>
+          <t>전복 글로벌 수입 시장 규모</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>누적 총 무역액</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>$148.50M</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>전복 글로벌 수입 시장 규모</t>
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>평균 수출입 단가</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>$32.40 / kg</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>전체 미수(Size) 평균 단가</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>평균 수출입 단가</t>
+          <t>최대 수입국 점유율 (일본)</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>$32.40 / kg</t>
+          <t>35.4%</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>전체 미수(Size) 평균 단가</t>
+          <t>완도산 활전복 항공/페리 1차 도매 수입</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>최대 수입국 점유율 (일본)</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>35.4%</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>완도산 활전복 항공/페리 1차 도매 수입</t>
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>최대 냉동 수입국 (미국)</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>42.1%</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>미 서부/동부 아시안 마트 냉동 IQF 해상 수입</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>최대 냉동 수입국 (미국)</t>
+          <t>최대 가공 수입국 (홍콩)</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>42.1%</t>
+          <t>48.5%</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>미 서부/동부 아시안 마트 냉동 IQF 해상 수입</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>최대 가공 수입국 (홍콩)</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>48.5%</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>홍콩 셩완 시장 명절 선물용 캔 통조림 수입</t>
         </is>
@@ -623,12 +618,12 @@
   <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="61.5" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="19.5" customWidth="1" min="4" max="4"/>
-    <col width="31.5" customWidth="1" min="5" max="5"/>
-    <col width="33" customWidth="1" min="6" max="6"/>
+    <col width="57.4" customWidth="1" min="1" max="1"/>
+    <col width="16.8" customWidth="1" min="2" max="2"/>
+    <col width="19.6" customWidth="1" min="3" max="3"/>
+    <col width="18.2" customWidth="1" min="4" max="4"/>
+    <col width="29.4" customWidth="1" min="5" max="5"/>
+    <col width="30.8" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -640,64 +635,64 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>품목 규격 / 미수</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>마리당 중량 범위</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>주요 수출 국가</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>평균 단가 ($/kg)</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>주요 타깃 시장 &amp; 바이어 채널</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>1인 상사 소싱 추천 포인트</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>10미 미만 (대과)</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>100g 이상 / 마리</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>한국 완도, 호주, 멕시코</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>$42.0 ~ $48.0</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>일본 고급 일식집, 스시야, 료칸</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>고급 항공직송 프리미엄 오퍼</t>
         </is>
@@ -736,32 +731,32 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>13 ~ 15미 (중과)</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>65g ~ 80g</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>한국, 중국</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>$30.0 ~ $34.0</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>관서 지역 레스토랑, 아시안 마트</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>H-Mart, 99 Ranch 채널 공급</t>
         </is>
@@ -800,34 +795,1012 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>20미 이상 (소과/가공)</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>50g 미만</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>한국, 중국</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>$18.0 ~ $22.0</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>통조림 가공, HMR 파우치 가공</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>통조림 FDA 승인 공장 연동</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="58.8" customWidth="1" min="1" max="1"/>
+    <col width="22.4" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="29.4" customWidth="1" min="4" max="4"/>
+    <col width="39.2" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>🗺️ [표 1] HS 0307.81 (활/신선 전복) TOP 10 유망 국가</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>유망순위</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>타깃 국가</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>무역액 점유율</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>컨택해야 할 로컬 파트너 종류</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>1인 상사 시장개척 포인트</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>1위</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>일본 (Japan)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>35.4%</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>도쿄 도요스 시장 수산물 수입 도매상사</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>완도산 활전복 페리/항공 직송 1차 수입 도매 공급</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>2위</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>중국 (China)</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>24.1%</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>동해안 수산물 수입 및 유통 상사</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>산둥성/상하이 고급 호텔 및 외식 체인 공급</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>3위</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>홍콩 (Hong Kong)</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>18.2%</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>고급 수산물 건재 시장 수입상사</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>고급 딤섬 및 레스토랑 직송 공급</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>4위</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>대만 (Taiwan)</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>7.5%</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>타이베이 고급 수산물 1차 수입상</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>일식 뷔페 및 연회장 활전복 대량 공급</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>5위</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>미국 (USA)</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>4.8%</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>LA/NY 아시안 수산물 벤더</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>한인/아시안 고소득층 대상 항공 직송</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>6위</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>싱가포르 (Singapore)</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>3.2%</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>마리나 베이 외식 그룹 벤더</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>고급 해산물 뷔페 및 호텔 공급</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>7위</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>베트남 (Vietnam)</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>2.5%</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>호치민/하노이 수산물 수입상</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>한국 식당가 및 고급 수산 레스토랑</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>8위</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>캐나다 (Canada)</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>1.8%</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>밴쿠버 아시안 수산 유통사</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>밴쿠버/토론토 아시안 마트 활전복</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>9위</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>태국 (Thailand)</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>1.3%</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>방콕 고급 수산물 수입 대리점</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>방콕 5성급 호텔 수산물 오퍼</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>10위</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>호주 (Australia)</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>1.2%</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>시드니 아시안 식품 유통 벤더</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>호주 한인 마트 및 아시안 레스토랑</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="56" customWidth="1" min="1" max="1"/>
+    <col width="26.6" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="37.8" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>🗺️ [표 2] HS 0307.83 (냉동 전복) TOP 10 유망 국가</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>유망순위</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>타깃 국가</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>무역액 점유율</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>컨택해야 할 로컬 파트너 종류</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>1인 상사 시장개척 포인트</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>1위</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>미국 (USA)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>42.1%</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>미 서부 최대 수산물 수입 벤더 (PASCO 등)</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>아시안 마트향 냉동 IQF 해상 컨테이너 공급</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>2위</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>대만 (Taiwan)</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>19.8%</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>타이베이 식자재 수입 디스트리뷰터</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>외식 뷔페 및 연회장향 IQF 냉동 대량 공급</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>3위</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>일본 (Japan)</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>15.3%</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>관서 지역 냉동 수산물 수입 대리점</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>성수기 외식 체인 원료 공급</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>4위</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>홍콩 (Hong Kong)</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>8.2%</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>냉동 수산물 전문 수입 유통사</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>외식 체인 및 호텔 냉동 IQF 공급</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>5위</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>싱가포르 (Singapore)</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>4.5%</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>동남아 아시안 식자재 유통 벤더</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>뷔페 및 딤섬 프랜차이즈 공급</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>6위</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>중국 (China)</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>3.8%</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>연안 도시 식품 가공 및 유통사</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>가공 원료용 냉동 IQF 전복 공급</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>7위</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>캐나다 (Canada)</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>2.1%</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>토론토 수산물 수입 벤더</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>아시안 마트 냉동 해산물 코너 공급</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>8위</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>베트남 (Vietnam)</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>1.8%</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>외식 식자재 1차 수입상</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>프랜차이즈 레스토랑 IQF 전복 공급</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>9위</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>태국 (Thailand)</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>1.3%</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>방콕 식자재 수입 대리점</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>외식 뷔페 및 씨푸드 레스토랑 공급</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>10위</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>영국 (United Kingdom)</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>1.1%</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>런던 아시안 식품 수입 벤더</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>런던 아시안 마트 및 한식당 공급</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="57.4" customWidth="1" min="1" max="1"/>
+    <col width="26.6" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="33.59999999999999" customWidth="1" min="4" max="4"/>
+    <col width="33.59999999999999" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>🗺️ [표 3] HS 1605.57 (전복 통조림) TOP 10 유망 국가</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>유망순위</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>타깃 국가</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>무역액 점유율</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>컨택해야 할 로컬 파트너 종류</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>1인 상사 시장개척 포인트</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>1위</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>홍콩 (Hong Kong)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>48.5%</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>홍콩 셩완 수산물 건재 시장 수입상사</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>춘절 명절 선물 세트용 B2B 캔 대량 공급</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>2위</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>싱가포르 (Singapore)</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>22.1%</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>싱가포르 고급 선물 세트 수입 유통 벤더</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>명절/기념일 프리미엄 선물용 캔 공급</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>3위</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>미국 (USA)</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>14.8%</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>북미 아시안 식품 수입 벤더 (아씨마켓 등)</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>FDA LACF 승인 캔 통조림 전역 유통</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>4위</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>대만 (Taiwan)</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>4.2%</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>명절 선물 세트 수입 유통사</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>명절 고급 전복 캔 선물 세트 공급</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>5위</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>캐나다 (Canada)</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>3.1%</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>밴쿠버 아시안 마트 유통 벤더</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>북미 한인/중국인 마트 캔 전복 공급</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>6위</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>호주 (Australia)</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>2.3%</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>시드니/멜버른 아시안 식품 수입상</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>선물용 캔 전복 유통</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>7위</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>일본 (Japan)</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>1.8%</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>고급 통조림 식자재 유통사</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>료칸 및 기프트 숍 고급 캔 오퍼</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>8위</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>베트남 (Vietnam)</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>1.2%</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>고급 선물 세트 수입상</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>호치민/하노이 명절 선물용 캔 전복</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>9위</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>태국 (Thailand)</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>1.1%</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>방콕 아시안 식품 수입 벤더</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>고급 아시안 마트 캔 유통</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>10위</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>영국 (United Kingdom)</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>0.9%</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>런던 프리미엄 기프트 숍 벤더</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>런던 아시안 명절 기프트 공급</t>
         </is>
       </c>
     </row>

</xml_diff>